<commit_message>
Add cold coffee and avocado pistachio toast menu items
</commit_message>
<xml_diff>
--- a/L_Cafe_Menu_Content.xlsx
+++ b/L_Cafe_Menu_Content.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R50acad6147624965"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="2" r:id="R5fc4b4c425bc4874"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="3" r:id="R0f4715bb6e284979"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="4" r:id="R7dd414b343d14fe6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ItemCodes" sheetId="5" r:id="Rccd0aa3acc4144f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R3ddad48ad4c54274"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categories" sheetId="2" r:id="Rdad087629b5e4f80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="3" r:id="Rc0f2b93226734f54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="4" r:id="R4a6e6c33e99b49b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ItemCodes" sheetId="5" r:id="R3f57a23a74ce4d8f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -474,7 +474,7 @@
         <x:v>counts</x:v>
       </x:c>
       <x:c r="B9" s="11" t="str">
-        <x:v>14 categories; 96 items; 19 options; 88 item-code rows.</x:v>
+        <x:v>14 categories; 101 items; 19 options; 93 item-code rows.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="31.5" customHeight="1">
@@ -488,7 +488,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raeabb2eebd5244a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40d90f2582f649bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -762,7 +762,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c82ddebcf4444f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4d43d8d11bc4e1d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4053,10 +4053,165 @@
       <x:c r="J97" s="10" t="str"/>
       <x:c r="K97" s="10" t="str"/>
     </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="str">
+        <x:v>menu-cold-coffee-06</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>slotId</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>cat-cold-coffee</x:v>
+      </x:c>
+      <x:c r="D98" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E98" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F98" t="str">
+        <x:v>آیس پرشین کافی پسته</x:v>
+      </x:c>
+      <x:c r="G98"/>
+      <x:c r="H98" t="str">
+        <x:v>۴۹۰</x:v>
+      </x:c>
+      <x:c r="I98" t="str">
+        <x:v>عکس آیس پرشین کافی پسته</x:v>
+      </x:c>
+      <x:c r="J98"/>
+      <x:c r="K98" t="str">
+        <x:v>menu-cold-coffee-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" t="str">
+        <x:v>menu-cold-coffee-07</x:v>
+      </x:c>
+      <x:c r="B99" t="str">
+        <x:v>slotId</x:v>
+      </x:c>
+      <x:c r="C99" t="str">
+        <x:v>cat-cold-coffee</x:v>
+      </x:c>
+      <x:c r="D99" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E99" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F99" t="str">
+        <x:v>آیس چاکلت</x:v>
+      </x:c>
+      <x:c r="G99"/>
+      <x:c r="H99" t="str">
+        <x:v>۳۸۰</x:v>
+      </x:c>
+      <x:c r="I99" t="str">
+        <x:v>عکس آیس چاکلت</x:v>
+      </x:c>
+      <x:c r="J99"/>
+      <x:c r="K99" t="str">
+        <x:v>menu-cold-coffee-07</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" t="str">
+        <x:v>menu-cold-coffee-08</x:v>
+      </x:c>
+      <x:c r="B100" t="str">
+        <x:v>slotId</x:v>
+      </x:c>
+      <x:c r="C100" t="str">
+        <x:v>cat-cold-coffee</x:v>
+      </x:c>
+      <x:c r="D100" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E100" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F100" t="str">
+        <x:v>آیس موکا 60</x:v>
+      </x:c>
+      <x:c r="G100"/>
+      <x:c r="H100" t="str">
+        <x:v>۴۰۰</x:v>
+      </x:c>
+      <x:c r="I100" t="str">
+        <x:v>عکس آیس موکا 60</x:v>
+      </x:c>
+      <x:c r="J100"/>
+      <x:c r="K100" t="str">
+        <x:v>menu-cold-coffee-08</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" t="str">
+        <x:v>menu-cold-coffee-09</x:v>
+      </x:c>
+      <x:c r="B101" t="str">
+        <x:v>slotId</x:v>
+      </x:c>
+      <x:c r="C101" t="str">
+        <x:v>cat-cold-coffee</x:v>
+      </x:c>
+      <x:c r="D101" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E101" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F101" t="str">
+        <x:v>آیس موکا 100</x:v>
+      </x:c>
+      <x:c r="G101"/>
+      <x:c r="H101" t="str">
+        <x:v>۴۲۰</x:v>
+      </x:c>
+      <x:c r="I101" t="str">
+        <x:v>عکس آیس موکا 100</x:v>
+      </x:c>
+      <x:c r="J101"/>
+      <x:c r="K101" t="str">
+        <x:v>menu-cold-coffee-09</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="A102" t="str">
+        <x:v>menu-food-09</x:v>
+      </x:c>
+      <x:c r="B102" t="str">
+        <x:v>slotId</x:v>
+      </x:c>
+      <x:c r="C102" t="str">
+        <x:v>cat-food</x:v>
+      </x:c>
+      <x:c r="D102" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E102" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F102" t="str">
+        <x:v>تست آووکادو پسته</x:v>
+      </x:c>
+      <x:c r="G102"/>
+      <x:c r="H102" t="str">
+        <x:v>۷۳۰</x:v>
+      </x:c>
+      <x:c r="I102" t="str">
+        <x:v>عکس تست آووکادو پسته</x:v>
+      </x:c>
+      <x:c r="J102"/>
+      <x:c r="K102" t="str">
+        <x:v>menu-food-09</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d3c1aa8ddc14b2e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dac3c0ce17c4656"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4476,7 +4631,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e7d828b61f943f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4de520f93524d4d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6005,10 +6160,95 @@
         <x:v>codes</x:v>
       </x:c>
     </x:row>
+    <x:row r="90">
+      <x:c r="A90" t="str">
+        <x:v>menu-cold-coffee-06::code-01</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>menu-cold-coffee-06</x:v>
+      </x:c>
+      <x:c r="C90" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D90" t="str">
+        <x:v>26015</x:v>
+      </x:c>
+      <x:c r="E90" t="str">
+        <x:v>code</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" t="str">
+        <x:v>menu-cold-coffee-07::code-01</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>menu-cold-coffee-07</x:v>
+      </x:c>
+      <x:c r="C91" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D91" t="str">
+        <x:v>26016</x:v>
+      </x:c>
+      <x:c r="E91" t="str">
+        <x:v>code</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" t="str">
+        <x:v>menu-cold-coffee-08::code-01</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>menu-cold-coffee-08</x:v>
+      </x:c>
+      <x:c r="C92" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D92" t="str">
+        <x:v>26010</x:v>
+      </x:c>
+      <x:c r="E92" t="str">
+        <x:v>code</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" t="str">
+        <x:v>menu-cold-coffee-09::code-01</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>menu-cold-coffee-09</x:v>
+      </x:c>
+      <x:c r="C93" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D93" t="str">
+        <x:v>26011</x:v>
+      </x:c>
+      <x:c r="E93" t="str">
+        <x:v>code</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>menu-food-09::code-01</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>menu-food-09</x:v>
+      </x:c>
+      <x:c r="C94" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D94" t="str">
+        <x:v>20014</x:v>
+      </x:c>
+      <x:c r="E94" t="str">
+        <x:v>code</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe3e85e670ef4d14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra46c56d9fad84aaf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>